<commit_message>
feat: add governed OpenAI provider gate
</commit_message>
<xml_diff>
--- a/specification/04_Matrices_y_Costos_v1.1(1).xlsx
+++ b/specification/04_Matrices_y_Costos_v1.1(1).xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readme" sheetId="1" r:id="R46d84e3970cb4580"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R797b1b5c82d6422a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Prices" sheetId="3" r:id="Rcd3f7ca8f47b4db5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Call Profile" sheetId="4" r:id="Rc559f176cdf1468a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="5" r:id="Rbf721c3b24a64b9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Components" sheetId="6" r:id="Rea8f46a95b7c4d03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Matrix" sheetId="7" r:id="R0777a7e09e6f4ff7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Re66464e93be6409c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readme" sheetId="1" r:id="R851e288df91c4ab0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Re9c81804a2df4693"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Prices" sheetId="3" r:id="R5ea12a5c96674221"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Call Profile" sheetId="4" r:id="Rc07d49b17880474b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="5" r:id="R2564b3d80c434951"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Components" sheetId="6" r:id="Rf8e6b1c9be274740"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Matrix" sheetId="7" r:id="R3a7726a0faba477b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R29905537fb774d15"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1391,9 +1391,6 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="48672768"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
         <c:axId val="48672768"/>
@@ -1462,7 +1459,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb9da4e3f460c49d0"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf975305defdd41f7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2377,7 +2374,7 @@
     <x:mergeCell ref="A2:E3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R600a9f7a66c14634"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2cb803f02554415"/>
 </x:worksheet>
 </file>
 
@@ -2580,10 +2577,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J6" s="29" t="str">
-        <x:v>2026-07-17</x:v>
+        <x:v>2026-08-08</x:v>
       </x:c>
       <x:c r="K6" s="29" t="str">
-        <x:v>P03 and P06-P09/P11 initial route; reasoning effort is configured per prompt.</x:v>
+        <x:v>P03 and P06-P09/P11 route. Conservative ceiling uses 1/0.1/6; a lower official 0.2/0.02/1.2 surface was also observed on 2026-08-08, so verify project pricing before spend.</x:v>
       </x:c>
       <x:c r="L6" s="29" t="str">
         <x:v>https://developers.openai.com/api/docs/pricing</x:v>
@@ -2621,7 +2618,7 @@
         <x:v>2026-07-17</x:v>
       </x:c>
       <x:c r="K7" s="29" t="str">
-        <x:v>Not a default route. Use only after a measured advantage over Luna-high for the task.</x:v>
+        <x:v>Historical price reference only. Terra is not callable in the OpenAI real-provider gate.</x:v>
       </x:c>
       <x:c r="L7" s="29" t="str">
         <x:v>https://developers.openai.com/api/docs/pricing</x:v>
@@ -2656,10 +2653,10 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="J8" s="29" t="str">
-        <x:v>2026-07-17</x:v>
+        <x:v>2026-08-08</x:v>
       </x:c>
       <x:c r="K8" s="29" t="str">
-        <x:v>P01/P02 medium and P04/P05 high; regional and long-context rules still apply.</x:v>
+        <x:v>P01/P02 medium and P04/P05 high. Conservative 5/0.5/30 ceiling; long-context multipliers and project-tier limits still apply.</x:v>
       </x:c>
       <x:c r="L8" s="29" t="str">
         <x:v>https://developers.openai.com/api/docs/pricing</x:v>
@@ -2697,7 +2694,7 @@
         <x:v>2026-07-17</x:v>
       </x:c>
       <x:c r="K9" s="29" t="str">
-        <x:v>Historical price only; do not reuse as a Gemini 3.6 Flash quote or callable route.</x:v>
+        <x:v>Historical comparison only; this provider/model has no callable route or authorization in the OpenAI gate.</x:v>
       </x:c>
       <x:c r="L9" s="29" t="str">
         <x:v>https://ai.google.dev/gemini-api/docs/pricing</x:v>
@@ -2735,7 +2732,7 @@
         <x:v>2026-07-17</x:v>
       </x:c>
       <x:c r="K10" s="29" t="str">
-        <x:v>Cost-efficient extraction/routing benchmark.</x:v>
+        <x:v>Historical comparison only; this provider/model has no callable route or authorization in the OpenAI gate.</x:v>
       </x:c>
       <x:c r="L10" s="29" t="str">
         <x:v>https://ai.google.dev/gemini-api/docs/pricing</x:v>
@@ -2773,7 +2770,7 @@
         <x:v>2026-07-17</x:v>
       </x:c>
       <x:c r="K11" s="29" t="str">
-        <x:v>Preview; prompts &gt;200K have higher prices. Not recommended as pinned production default.</x:v>
+        <x:v>Historical comparison only; this provider/model has no callable route or authorization in the OpenAI gate.</x:v>
       </x:c>
       <x:c r="L11" s="29" t="str">
         <x:v>https://ai.google.dev/gemini-api/docs/pricing</x:v>
@@ -2811,7 +2808,7 @@
         <x:v>2026-07-17</x:v>
       </x:c>
       <x:c r="K12" s="29" t="str">
-        <x:v>Requires 30-day retention; exclude from ZDR tenants.</x:v>
+        <x:v>Historical comparison only; this provider/model has no callable route or authorization in the OpenAI gate.</x:v>
       </x:c>
       <x:c r="L12" s="29" t="str">
         <x:v>https://platform.claude.com/docs/en/about-claude/pricing</x:v>
@@ -2849,7 +2846,7 @@
         <x:v>2026-07-17</x:v>
       </x:c>
       <x:c r="K13" s="29" t="str">
-        <x:v>Complex-task benchmark; cache write shown at 1.25x for 5-minute cache.</x:v>
+        <x:v>Historical comparison only; this provider/model has no callable route or authorization in the OpenAI gate.</x:v>
       </x:c>
       <x:c r="L13" s="29" t="str">
         <x:v>https://platform.claude.com/docs/en/about-claude/pricing</x:v>
@@ -2887,7 +2884,7 @@
         <x:v>Through 2026-08-31</x:v>
       </x:c>
       <x:c r="K14" s="29" t="str">
-        <x:v>Intro price; published regular price becomes 3/15 input/output after promotion.</x:v>
+        <x:v>Historical comparison only; this provider/model has no callable route or authorization in the OpenAI gate.</x:v>
       </x:c>
       <x:c r="L14" s="29" t="str">
         <x:v>https://platform.claude.com/docs/en/about-claude/pricing</x:v>
@@ -2925,7 +2922,7 @@
         <x:v>2026-07-17</x:v>
       </x:c>
       <x:c r="K15" s="32" t="str">
-        <x:v>Fast/low-cost comparison; 200K context, lower output limit than top models.</x:v>
+        <x:v>Historical comparison only; this provider/model has no callable route or authorization in the OpenAI gate.</x:v>
       </x:c>
       <x:c r="L15" s="32" t="str">
         <x:v>https://platform.claude.com/docs/en/about-claude/pricing</x:v>
@@ -2949,7 +2946,7 @@
         <x:v>Add before paid bake-off</x:v>
       </x:c>
       <x:c r="K16" s="241" t="str">
-        <x:v>Approved comparator for specific multimodal tasks only; obtain an official current price before costing.</x:v>
+        <x:v>Historical comparison only; this provider/model has no callable route or authorization in the OpenAI gate.</x:v>
       </x:c>
       <x:c r="L16" s="241" t="str">
         <x:v>https://ai.google.dev/gemini-api/docs/pricing</x:v>
@@ -3051,7 +3048,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>P01-P11 routes are explicit. The deterministic resolver checks capabilities and data policy before calls; P10 has zero frequency until its grounding/citation/abstention bake-off closes.</x:v>
+        <x:v>Only P01-P09 and P11 have explicit OpenAI routes in this gate. P10 is disabled with zero frequency; Terra and non-OpenAI rows are historical references, never callable fallbacks.</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
         <x:v>Each row represents a pipeline task. Frequency multiplier models routing/escalation; batch share blends standard and batch prices. Price columns and costs are formulas.</x:v>
@@ -3854,7 +3851,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="R15" s="241" t="str">
-        <x:v>Disabled cost proxy only. Route remains an open bake-off; do not treat Luna as selected.</x:v>
+        <x:v>Disabled cost proxy only. P10 has zero frequency, no selected model, no callable route and no bake-off authorization in this gate.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
@@ -3918,7 +3915,7 @@
         <x:v>0.000715</x:v>
       </x:c>
       <x:c r="R16" s="241" t="str">
-        <x:v>Luna minimal, temperature 0; editable 5% structural-failure frequency.</x:v>
+        <x:v>Luna low (human-authorized replacement for historical minimal); desired temperature 0 is not sent because compatibility with GPT-5.6 reasoning is not currently documented. Editable 5% structural-failure frequency.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3940,7 +3937,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc53bf0b22aa54cd3"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fb7b0348f0b49e5"/>
 </x:worksheet>
 </file>
 
@@ -4751,8 +4748,8 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c096397649343c2"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cae69ba4f924303"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racc271c39f2740b9"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45b7b6519a794c43"/>
 </x:worksheet>
 </file>
 
@@ -5804,28 +5801,28 @@
         <x:v>P10 Enriched context</x:v>
       </x:c>
       <x:c r="B15" s="29" t="str">
-        <x:v>Open bake-off</x:v>
+        <x:v>DISABLED — no callable route</x:v>
       </x:c>
       <x:c r="C15" s="29" t="str">
-        <x:v>per approved route</x:v>
+        <x:v>n/a</x:v>
       </x:c>
       <x:c r="D15" s="29" t="str">
-        <x:v>low</x:v>
+        <x:v>not sent</x:v>
       </x:c>
       <x:c r="E15" s="29" t="str">
-        <x:v>Citations + relevant modality</x:v>
+        <x:v>Historical contract only</x:v>
       </x:c>
       <x:c r="F15" s="29" t="str">
-        <x:v>No generic fallback</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="G15" s="29" t="str">
-        <x:v>Native PDF/audio/video or measured task advantage</x:v>
+        <x:v>Blocked before transport</x:v>
       </x:c>
       <x:c r="H15" s="29" t="str">
-        <x:v>Approved task/modality/tenant/data</x:v>
+        <x:v>CVA_P10_ENABLED=false; no provider authorized</x:v>
       </x:c>
       <x:c r="I15" s="29" t="str">
-        <x:v>Grounding, citations, abstention</x:v>
+        <x:v>0 calls</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="68" customHeight="1">
@@ -5836,10 +5833,10 @@
         <x:v>GPT-5.6 Luna</x:v>
       </x:c>
       <x:c r="C16" s="29" t="str">
-        <x:v>minimal</x:v>
+        <x:v>low</x:v>
       </x:c>
       <x:c r="D16" s="29" t="str">
-        <x:v>0</x:v>
+        <x:v>not sent (desired 0)</x:v>
       </x:c>
       <x:c r="E16" s="29" t="str">
         <x:v>Structured JSON</x:v>
@@ -5862,28 +5859,28 @@
         <x:v>Gemini 3.6 Flash policy</x:v>
       </x:c>
       <x:c r="B17" s="29" t="str">
-        <x:v>Alternative only</x:v>
+        <x:v>Not callable in this gate</x:v>
       </x:c>
       <x:c r="C17" s="29" t="str">
-        <x:v>task-specific</x:v>
+        <x:v>n/a</x:v>
       </x:c>
       <x:c r="D17" s="29" t="str">
-        <x:v>low</x:v>
+        <x:v>not sent</x:v>
       </x:c>
       <x:c r="E17" s="29" t="str">
-        <x:v>Native video/audio/PDF where required</x:v>
+        <x:v>Historical reference only</x:v>
       </x:c>
       <x:c r="F17" s="29" t="str">
-        <x:v>Never automatic</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="G17" s="29" t="str">
-        <x:v>Unsupported modality or proven bake-off advantage</x:v>
+        <x:v>No eligibility in this gate</x:v>
       </x:c>
       <x:c r="H17" s="29" t="str">
-        <x:v>Explicit approval per task/modality/tenant/data</x:v>
+        <x:v>Non-OpenAI provider not authorized</x:v>
       </x:c>
       <x:c r="I17" s="29" t="str">
-        <x:v>Beat baseline on task</x:v>
+        <x:v>No evaluation in this gate</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="68" customHeight="1">
@@ -5891,28 +5888,28 @@
         <x:v>Terra policy</x:v>
       </x:c>
       <x:c r="B18" s="32" t="str">
-        <x:v>Alternative only</x:v>
+        <x:v>Not callable in this gate</x:v>
       </x:c>
       <x:c r="C18" s="32" t="str">
-        <x:v>measured</x:v>
+        <x:v>n/a</x:v>
       </x:c>
       <x:c r="D18" s="32" t="str">
-        <x:v>low</x:v>
+        <x:v>not sent</x:v>
       </x:c>
       <x:c r="E18" s="32" t="str">
-        <x:v>Declared route capabilities</x:v>
+        <x:v>Historical reference only</x:v>
       </x:c>
       <x:c r="F18" s="32" t="str">
-        <x:v>Never default</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="G18" s="32" t="str">
-        <x:v>Measured advantage over Luna-high</x:v>
+        <x:v>No eligibility in this gate</x:v>
       </x:c>
       <x:c r="H18" s="32" t="str">
-        <x:v>Same pre-call policy checks</x:v>
+        <x:v>Terra excluded by the binding route matrix</x:v>
       </x:c>
       <x:c r="I18" s="32" t="str">
-        <x:v>Statistically/materially better</x:v>
+        <x:v>No evaluation in this gate</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Implement LUNA_BASELINE_V1 provider profile
</commit_message>
<xml_diff>
--- a/specification/04_Matrices_y_Costos_v1.1(1).xlsx
+++ b/specification/04_Matrices_y_Costos_v1.1(1).xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readme" sheetId="1" r:id="R851e288df91c4ab0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Re9c81804a2df4693"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Prices" sheetId="3" r:id="R5ea12a5c96674221"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Call Profile" sheetId="4" r:id="Rc07d49b17880474b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="5" r:id="R2564b3d80c434951"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Components" sheetId="6" r:id="Rf8e6b1c9be274740"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Matrix" sheetId="7" r:id="R3a7726a0faba477b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R29905537fb774d15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readme" sheetId="1" r:id="R58d5071e96ca4d61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R70bbee8e9b574435"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Prices" sheetId="3" r:id="R65f87085ed054e5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Call Profile" sheetId="4" r:id="R7ca0c4c6d664471b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="5" r:id="R72ba9483dc9947b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Components" sheetId="6" r:id="R1c72e07694874f2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Matrix" sheetId="7" r:id="R001aa577f3814f40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R8909fd2d9c494bb9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1459,7 +1459,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf975305defdd41f7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9483595450a24955"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1723,7 +1723,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>Companion workbook for the cloud experimental MVP and future architecture. Pricing snapshot: 2026-07-17; design revision: 2026-07-30. Blue cells are editable assumptions.</x:v>
+        <x:v>Companion workbook for the cloud experimental MVP and future architecture. Pricing snapshot: 2026-08-08; route revision: 2026-08-08. Blue cells are editable assumptions.</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
         <x:v>Companion workbook for the comprehension-verification assessment architecture. Pricing snapshot: 2026-07-17. All currency values are USD and all assumptions in blue cells are editable.</x:v>
@@ -1968,7 +1968,7 @@
         <x:v>Call Profile</x:v>
       </x:c>
       <x:c r="B21" s="29" t="str">
-        <x:v>P01-P11 token/caching profile using the approved Sol/Luna matrix; P10 remains disabled until bake-off.</x:v>
+        <x:v>P01-P09/P11 token and cost profile for LUNA_BASELINE_V1; the mixed Sol/Luna matrix is historical only and P10 remains disabled.</x:v>
       </x:c>
       <x:c r="C21" s="29" t="str"/>
       <x:c r="D21" s="29" t="str"/>
@@ -2374,7 +2374,7 @@
     <x:mergeCell ref="A2:E3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2cb803f02554415"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c9c040d101e4141"/>
 </x:worksheet>
 </file>
 
@@ -2556,31 +2556,31 @@
         <x:v>OpenAI</x:v>
       </x:c>
       <x:c r="C6" s="70" t="n">
-        <x:v>1</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="D6" s="70" t="n">
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="E6" s="70" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="F6" s="70" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="G6" s="70" t="n">
         <x:v>0.1</x:v>
       </x:c>
-      <x:c r="E6" s="70" t="n">
-        <x:v>1.25</x:v>
-      </x:c>
-      <x:c r="F6" s="70" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="G6" s="70" t="n">
-        <x:v>0.5</x:v>
-      </x:c>
       <x:c r="H6" s="70" t="n">
-        <x:v>0.05</x:v>
+        <x:v>0.01</x:v>
       </x:c>
       <x:c r="I6" s="70" t="n">
-        <x:v>3</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="J6" s="29" t="str">
         <x:v>2026-08-08</x:v>
       </x:c>
       <x:c r="K6" s="29" t="str">
-        <x:v>P03 and P06-P09/P11 route. Conservative ceiling uses 1/0.1/6; a lower official 0.2/0.02/1.2 surface was also observed on 2026-08-08, so verify project pricing before spend.</x:v>
+        <x:v>Active LUNA_BASELINE_V1 price: Standard short-context 0.20/0.02/0.25/1.20. Batch reference 0.10/0.01/0.60; active calls use service_tier=default and 0% Batch.</x:v>
       </x:c>
       <x:c r="L6" s="29" t="str">
         <x:v>https://developers.openai.com/api/docs/pricing</x:v>
@@ -2656,7 +2656,7 @@
         <x:v>2026-08-08</x:v>
       </x:c>
       <x:c r="K8" s="29" t="str">
-        <x:v>P01/P02 medium and P04/P05 high. Conservative 5/0.5/30 ceiling; long-context multipliers and project-tier limits still apply.</x:v>
+        <x:v>Historical comparison candidate only. Sol has no active, fallback or automatically callable route in LUNA_BASELINE_V1.</x:v>
       </x:c>
       <x:c r="L8" s="29" t="str">
         <x:v>https://developers.openai.com/api/docs/pricing</x:v>
@@ -3048,7 +3048,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>Only P01-P09 and P11 have explicit OpenAI routes in this gate. P10 is disabled with zero frequency; Terra and non-OpenAI rows are historical references, never callable fallbacks.</x:v>
+        <x:v>LUNA_BASELINE_V1 uses only GPT-5.6 Luna for P01-P09/P11. P10 has zero frequency/no callable route; the mixed Sol/Luna matrix is historical and never a fallback.</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
         <x:v>Each row represents a pipeline task. Frequency multiplier models routing/escalation; batch share blends standard and batch prices. Price columns and costs are formulas.</x:v>
@@ -3222,7 +3222,7 @@
         <x:v>ACTIVITY</x:v>
       </x:c>
       <x:c r="C6" s="74" t="str">
-        <x:v>GPT-5.6 Sol</x:v>
+        <x:v>GPT-5.6 Luna</x:v>
       </x:c>
       <x:c r="D6" s="80" t="n">
         <x:v>1</x:v>
@@ -3244,38 +3244,38 @@
       </x:c>
       <x:c r="J6" s="84" t="n">
         <x:f>VLOOKUP(C6,'Model Prices'!$A$6:$I$15,3,FALSE)</x:f>
-        <x:v>5</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="K6" s="84" t="n">
         <x:f>VLOOKUP(C6,'Model Prices'!$A$6:$I$15,4,FALSE)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.02</x:v>
       </x:c>
       <x:c r="L6" s="84" t="n">
         <x:f>VLOOKUP(C6,'Model Prices'!$A$6:$I$15,6,FALSE)</x:f>
-        <x:v>30</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="M6" s="84" t="n">
         <x:f>VLOOKUP(C6,'Model Prices'!$A$6:$I$15,7,FALSE)</x:f>
-        <x:v>2.5</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="N6" s="84" t="n">
         <x:f>VLOOKUP(C6,'Model Prices'!$A$6:$I$15,8,FALSE)</x:f>
-        <x:v>0.25</x:v>
+        <x:v>0.01</x:v>
       </x:c>
       <x:c r="O6" s="84" t="n">
         <x:f>VLOOKUP(C6,'Model Prices'!$A$6:$I$15,9,FALSE)</x:f>
-        <x:v>15</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="P6" s="84" t="n">
         <x:f>(E6*(1-F6)/'Assumptions'!$B$6)*(J6*(1-H6)+M6*H6)+(E6*F6/'Assumptions'!$B$6)*(K6*(1-H6)+N6*H6)+(G6/'Assumptions'!$B$6)*(L6*(1-H6)+O6*H6)</x:f>
-        <x:v>0.1392</x:v>
+        <x:v>0.005568</x:v>
       </x:c>
       <x:c r="Q6" s="84" t="n">
         <x:f>D6*I6*P6*(1+'Assumptions'!$B$13)*(1+'Assumptions'!$B$14)</x:f>
-        <x:v>0.1392</x:v>
+        <x:v>0.005568</x:v>
       </x:c>
       <x:c r="R6" s="29" t="str">
-        <x:v>Sol medium; one-time per approved activity.</x:v>
+        <x:v>Luna medium; one-time per approved activity.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="48" customHeight="1">
@@ -3286,7 +3286,7 @@
         <x:v>ACTIVITY</x:v>
       </x:c>
       <x:c r="C7" s="74" t="str">
-        <x:v>GPT-5.6 Sol</x:v>
+        <x:v>GPT-5.6 Luna</x:v>
       </x:c>
       <x:c r="D7" s="80" t="n">
         <x:v>1</x:v>
@@ -3308,38 +3308,38 @@
       </x:c>
       <x:c r="J7" s="84" t="n">
         <x:f>VLOOKUP(C7,'Model Prices'!$A$6:$I$15,3,FALSE)</x:f>
-        <x:v>5</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="K7" s="84" t="n">
         <x:f>VLOOKUP(C7,'Model Prices'!$A$6:$I$15,4,FALSE)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.02</x:v>
       </x:c>
       <x:c r="L7" s="84" t="n">
         <x:f>VLOOKUP(C7,'Model Prices'!$A$6:$I$15,6,FALSE)</x:f>
-        <x:v>30</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="M7" s="84" t="n">
         <x:f>VLOOKUP(C7,'Model Prices'!$A$6:$I$15,7,FALSE)</x:f>
-        <x:v>2.5</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="N7" s="84" t="n">
         <x:f>VLOOKUP(C7,'Model Prices'!$A$6:$I$15,8,FALSE)</x:f>
-        <x:v>0.25</x:v>
+        <x:v>0.01</x:v>
       </x:c>
       <x:c r="O7" s="84" t="n">
         <x:f>VLOOKUP(C7,'Model Prices'!$A$6:$I$15,9,FALSE)</x:f>
-        <x:v>15</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="P7" s="84" t="n">
         <x:f>(E7*(1-F7)/'Assumptions'!$B$6)*(J7*(1-H7)+M7*H7)+(E7*F7/'Assumptions'!$B$6)*(K7*(1-H7)+N7*H7)+(G7/'Assumptions'!$B$6)*(L7*(1-H7)+O7*H7)</x:f>
-        <x:v>0.1042</x:v>
+        <x:v>0.004168</x:v>
       </x:c>
       <x:c r="Q7" s="84" t="n">
         <x:f>D7*I7*P7*(1+'Assumptions'!$B$13)*(1+'Assumptions'!$B$14)</x:f>
-        <x:v>0.1042</x:v>
+        <x:v>0.004168</x:v>
       </x:c>
       <x:c r="R7" s="29" t="str">
-        <x:v>Sol medium; preserves grading weight separately.</x:v>
+        <x:v>Luna medium; preserves grading weight separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
@@ -3372,35 +3372,35 @@
       </x:c>
       <x:c r="J8" s="84" t="n">
         <x:f>VLOOKUP(C8,'Model Prices'!$A$6:$I$15,3,FALSE)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="K8" s="84" t="n">
         <x:f>VLOOKUP(C8,'Model Prices'!$A$6:$I$15,4,FALSE)</x:f>
-        <x:v>0.1</x:v>
+        <x:v>0.02</x:v>
       </x:c>
       <x:c r="L8" s="84" t="n">
         <x:f>VLOOKUP(C8,'Model Prices'!$A$6:$I$15,6,FALSE)</x:f>
-        <x:v>6</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="M8" s="84" t="n">
         <x:f>VLOOKUP(C8,'Model Prices'!$A$6:$I$15,7,FALSE)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="N8" s="84" t="n">
         <x:f>VLOOKUP(C8,'Model Prices'!$A$6:$I$15,8,FALSE)</x:f>
-        <x:v>0.05</x:v>
+        <x:v>0.01</x:v>
       </x:c>
       <x:c r="O8" s="84" t="n">
         <x:f>VLOOKUP(C8,'Model Prices'!$A$6:$I$15,9,FALSE)</x:f>
-        <x:v>3</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="P8" s="84" t="n">
         <x:f>(E8*(1-F8)/'Assumptions'!$B$6)*(J8*(1-H8)+M8*H8)+(E8*F8/'Assumptions'!$B$6)*(K8*(1-H8)+N8*H8)+(G8/'Assumptions'!$B$6)*(L8*(1-H8)+O8*H8)</x:f>
-        <x:v>0.0152525</x:v>
+        <x:v>0.0030505</x:v>
       </x:c>
       <x:c r="Q8" s="84" t="n">
         <x:f>D8*I8*P8*(1+'Assumptions'!$B$13)*(1+'Assumptions'!$B$14)</x:f>
-        <x:v>0.0152525</x:v>
+        <x:v>0.0030505</x:v>
       </x:c>
       <x:c r="R8" s="29" t="str">
         <x:v>Luna high; groups/explains issues and never decides for the teacher.</x:v>
@@ -3414,7 +3414,7 @@
         <x:v>ACTIVITY</x:v>
       </x:c>
       <x:c r="C9" s="74" t="str">
-        <x:v>GPT-5.6 Sol</x:v>
+        <x:v>GPT-5.6 Luna</x:v>
       </x:c>
       <x:c r="D9" s="80" t="n">
         <x:v>1</x:v>
@@ -3436,38 +3436,38 @@
       </x:c>
       <x:c r="J9" s="84" t="n">
         <x:f>VLOOKUP(C9,'Model Prices'!$A$6:$I$15,3,FALSE)</x:f>
-        <x:v>5</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="K9" s="84" t="n">
         <x:f>VLOOKUP(C9,'Model Prices'!$A$6:$I$15,4,FALSE)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.02</x:v>
       </x:c>
       <x:c r="L9" s="84" t="n">
         <x:f>VLOOKUP(C9,'Model Prices'!$A$6:$I$15,6,FALSE)</x:f>
-        <x:v>30</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="M9" s="84" t="n">
         <x:f>VLOOKUP(C9,'Model Prices'!$A$6:$I$15,7,FALSE)</x:f>
-        <x:v>2.5</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="N9" s="84" t="n">
         <x:f>VLOOKUP(C9,'Model Prices'!$A$6:$I$15,8,FALSE)</x:f>
-        <x:v>0.25</x:v>
+        <x:v>0.01</x:v>
       </x:c>
       <x:c r="O9" s="84" t="n">
         <x:f>VLOOKUP(C9,'Model Prices'!$A$6:$I$15,9,FALSE)</x:f>
-        <x:v>15</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="P9" s="84" t="n">
         <x:f>(E9*(1-F9)/'Assumptions'!$B$6)*(J9*(1-H9)+M9*H9)+(E9*F9/'Assumptions'!$B$6)*(K9*(1-H9)+N9*H9)+(G9/'Assumptions'!$B$6)*(L9*(1-H9)+O9*H9)</x:f>
-        <x:v>0.17609999999999998</x:v>
+        <x:v>0.007044</x:v>
       </x:c>
       <x:c r="Q9" s="84" t="n">
         <x:f>D9*I9*P9*(1+'Assumptions'!$B$13)*(1+'Assumptions'!$B$14)</x:f>
-        <x:v>0.17609999999999998</x:v>
+        <x:v>0.007044</x:v>
       </x:c>
       <x:c r="R9" s="29" t="str">
-        <x:v>Sol high; catalog is independent of question_count.</x:v>
+        <x:v>Luna high; catalog remains independent of question_count.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
@@ -3478,7 +3478,7 @@
         <x:v>ACTIVITY</x:v>
       </x:c>
       <x:c r="C10" s="74" t="str">
-        <x:v>GPT-5.6 Sol</x:v>
+        <x:v>GPT-5.6 Luna</x:v>
       </x:c>
       <x:c r="D10" s="80" t="n">
         <x:v>1</x:v>
@@ -3500,38 +3500,38 @@
       </x:c>
       <x:c r="J10" s="84" t="n">
         <x:f>VLOOKUP(C10,'Model Prices'!$A$6:$I$15,3,FALSE)</x:f>
-        <x:v>5</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="K10" s="84" t="n">
         <x:f>VLOOKUP(C10,'Model Prices'!$A$6:$I$15,4,FALSE)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.02</x:v>
       </x:c>
       <x:c r="L10" s="84" t="n">
         <x:f>VLOOKUP(C10,'Model Prices'!$A$6:$I$15,6,FALSE)</x:f>
-        <x:v>30</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="M10" s="84" t="n">
         <x:f>VLOOKUP(C10,'Model Prices'!$A$6:$I$15,7,FALSE)</x:f>
-        <x:v>2.5</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="N10" s="84" t="n">
         <x:f>VLOOKUP(C10,'Model Prices'!$A$6:$I$15,8,FALSE)</x:f>
-        <x:v>0.25</x:v>
+        <x:v>0.01</x:v>
       </x:c>
       <x:c r="O10" s="84" t="n">
         <x:f>VLOOKUP(C10,'Model Prices'!$A$6:$I$15,9,FALSE)</x:f>
-        <x:v>15</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="P10" s="84" t="n">
         <x:f>(E10*(1-F10)/'Assumptions'!$B$6)*(J10*(1-H10)+M10*H10)+(E10*F10/'Assumptions'!$B$6)*(K10*(1-H10)+N10*H10)+(G10/'Assumptions'!$B$6)*(L10*(1-H10)+O10*H10)</x:f>
-        <x:v>0.10475</x:v>
+        <x:v>0.00419</x:v>
       </x:c>
       <x:c r="Q10" s="84" t="n">
         <x:f>D10*I10*P10*(1+'Assumptions'!$B$13)*(1+'Assumptions'!$B$14)</x:f>
-        <x:v>0.10475</x:v>
+        <x:v>0.00419</x:v>
       </x:c>
       <x:c r="R10" s="29" t="str">
-        <x:v>Sol high; independent critical review.</x:v>
+        <x:v>Luna high; independent critical review.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
@@ -3564,35 +3564,35 @@
       </x:c>
       <x:c r="J11" s="84" t="n">
         <x:f>VLOOKUP(C11,'Model Prices'!$A$6:$I$15,3,FALSE)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="K11" s="84" t="n">
         <x:f>VLOOKUP(C11,'Model Prices'!$A$6:$I$15,4,FALSE)</x:f>
-        <x:v>0.1</x:v>
+        <x:v>0.02</x:v>
       </x:c>
       <x:c r="L11" s="84" t="n">
         <x:f>VLOOKUP(C11,'Model Prices'!$A$6:$I$15,6,FALSE)</x:f>
-        <x:v>6</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="M11" s="84" t="n">
         <x:f>VLOOKUP(C11,'Model Prices'!$A$6:$I$15,7,FALSE)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="N11" s="84" t="n">
         <x:f>VLOOKUP(C11,'Model Prices'!$A$6:$I$15,8,FALSE)</x:f>
-        <x:v>0.05</x:v>
+        <x:v>0.01</x:v>
       </x:c>
       <x:c r="O11" s="84" t="n">
         <x:f>VLOOKUP(C11,'Model Prices'!$A$6:$I$15,9,FALSE)</x:f>
-        <x:v>3</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="P11" s="84" t="n">
         <x:f>(E11*(1-F11)/'Assumptions'!$B$6)*(J11*(1-H11)+M11*H11)+(E11*F11/'Assumptions'!$B$6)*(K11*(1-H11)+N11*H11)+(G11/'Assumptions'!$B$6)*(L11*(1-H11)+O11*H11)</x:f>
-        <x:v>0.0374</x:v>
+        <x:v>0.0074800000000000005</x:v>
       </x:c>
       <x:c r="Q11" s="84" t="n">
         <x:f>D11*I11*P11*(1+'Assumptions'!$B$13)*(1+'Assumptions'!$B$14)</x:f>
-        <x:v>0.0374</x:v>
+        <x:v>0.0074800000000000005</x:v>
       </x:c>
       <x:c r="R11" s="29" t="str">
         <x:v>Luna high; maps dimension, variant, evidence and opportunities.</x:v>
@@ -3628,35 +3628,35 @@
       </x:c>
       <x:c r="J12" s="84" t="n">
         <x:f>VLOOKUP(C12,'Model Prices'!$A$6:$I$15,3,FALSE)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="K12" s="84" t="n">
         <x:f>VLOOKUP(C12,'Model Prices'!$A$6:$I$15,4,FALSE)</x:f>
-        <x:v>0.1</x:v>
+        <x:v>0.02</x:v>
       </x:c>
       <x:c r="L12" s="84" t="n">
         <x:f>VLOOKUP(C12,'Model Prices'!$A$6:$I$15,6,FALSE)</x:f>
-        <x:v>6</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="M12" s="84" t="n">
         <x:f>VLOOKUP(C12,'Model Prices'!$A$6:$I$15,7,FALSE)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="N12" s="84" t="n">
         <x:f>VLOOKUP(C12,'Model Prices'!$A$6:$I$15,8,FALSE)</x:f>
-        <x:v>0.05</x:v>
+        <x:v>0.01</x:v>
       </x:c>
       <x:c r="O12" s="84" t="n">
         <x:f>VLOOKUP(C12,'Model Prices'!$A$6:$I$15,9,FALSE)</x:f>
-        <x:v>3</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="P12" s="84" t="n">
         <x:f>(E12*(1-F12)/'Assumptions'!$B$6)*(J12*(1-H12)+M12*H12)+(E12*F12/'Assumptions'!$B$6)*(K12*(1-H12)+N12*H12)+(G12/'Assumptions'!$B$6)*(L12*(1-H12)+O12*H12)</x:f>
-        <x:v>0.031275</x:v>
+        <x:v>0.006255</x:v>
       </x:c>
       <x:c r="Q12" s="84" t="n">
         <x:f>D12*I12*P12*(1+'Assumptions'!$B$13)*(1+'Assumptions'!$B$14)</x:f>
-        <x:v>0.031275</x:v>
+        <x:v>0.006255</x:v>
       </x:c>
       <x:c r="R12" s="29" t="str">
         <x:v>Luna high; one question per planned opportunity; scenarios scale by question count.</x:v>
@@ -3692,35 +3692,35 @@
       </x:c>
       <x:c r="J13" s="84" t="n">
         <x:f>VLOOKUP(C13,'Model Prices'!$A$6:$I$15,3,FALSE)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="K13" s="84" t="n">
         <x:f>VLOOKUP(C13,'Model Prices'!$A$6:$I$15,4,FALSE)</x:f>
-        <x:v>0.1</x:v>
+        <x:v>0.02</x:v>
       </x:c>
       <x:c r="L13" s="84" t="n">
         <x:f>VLOOKUP(C13,'Model Prices'!$A$6:$I$15,6,FALSE)</x:f>
-        <x:v>6</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="M13" s="84" t="n">
         <x:f>VLOOKUP(C13,'Model Prices'!$A$6:$I$15,7,FALSE)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="N13" s="84" t="n">
         <x:f>VLOOKUP(C13,'Model Prices'!$A$6:$I$15,8,FALSE)</x:f>
-        <x:v>0.05</x:v>
+        <x:v>0.01</x:v>
       </x:c>
       <x:c r="O13" s="84" t="n">
         <x:f>VLOOKUP(C13,'Model Prices'!$A$6:$I$15,9,FALSE)</x:f>
-        <x:v>3</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="P13" s="84" t="n">
         <x:f>(E13*(1-F13)/'Assumptions'!$B$6)*(J13*(1-H13)+M13*H13)+(E13*F13/'Assumptions'!$B$6)*(K13*(1-H13)+N13*H13)+(G13/'Assumptions'!$B$6)*(L13*(1-H13)+O13*H13)</x:f>
-        <x:v>0.0205</x:v>
+        <x:v>0.0041</x:v>
       </x:c>
       <x:c r="Q13" s="84" t="n">
         <x:f>D13*I13*P13*(1+'Assumptions'!$B$13)*(1+'Assumptions'!$B$14)</x:f>
-        <x:v>0.0205</x:v>
+        <x:v>0.0041</x:v>
       </x:c>
       <x:c r="R13" s="29" t="str">
         <x:v>Luna high; independent prompt plus deterministic vetoes.</x:v>
@@ -3756,35 +3756,35 @@
       </x:c>
       <x:c r="J14" s="85" t="n">
         <x:f>VLOOKUP(C14,'Model Prices'!$A$6:$I$15,3,FALSE)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="K14" s="85" t="n">
         <x:f>VLOOKUP(C14,'Model Prices'!$A$6:$I$15,4,FALSE)</x:f>
-        <x:v>0.1</x:v>
+        <x:v>0.02</x:v>
       </x:c>
       <x:c r="L14" s="85" t="n">
         <x:f>VLOOKUP(C14,'Model Prices'!$A$6:$I$15,6,FALSE)</x:f>
-        <x:v>6</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="M14" s="85" t="n">
         <x:f>VLOOKUP(C14,'Model Prices'!$A$6:$I$15,7,FALSE)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="N14" s="85" t="n">
         <x:f>VLOOKUP(C14,'Model Prices'!$A$6:$I$15,8,FALSE)</x:f>
-        <x:v>0.05</x:v>
+        <x:v>0.01</x:v>
       </x:c>
       <x:c r="O14" s="85" t="n">
         <x:f>VLOOKUP(C14,'Model Prices'!$A$6:$I$15,9,FALSE)</x:f>
-        <x:v>3</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="P14" s="85" t="n">
         <x:f>(E14*(1-F14)/'Assumptions'!$B$6)*(J14*(1-H14)+M14*H14)+(E14*F14/'Assumptions'!$B$6)*(K14*(1-H14)+N14*H14)+(G14/'Assumptions'!$B$6)*(L14*(1-H14)+O14*H14)</x:f>
-        <x:v>0.01528</x:v>
+        <x:v>0.003056</x:v>
       </x:c>
       <x:c r="Q14" s="85" t="n">
         <x:f>D14*I14*P14*(1+'Assumptions'!$B$13)*(1+'Assumptions'!$B$14)</x:f>
-        <x:v>0.01528</x:v>
+        <x:v>0.003056</x:v>
       </x:c>
       <x:c r="R14" s="32" t="str">
         <x:v>Luna high; structured guide stored in platform.</x:v>
@@ -3820,31 +3820,31 @@
       </x:c>
       <x:c r="J15" s="249" t="n">
         <x:f>VLOOKUP(C15,'Model Prices'!$A$6:$I$15,3,FALSE)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="K15" s="249" t="n">
         <x:f>VLOOKUP(C15,'Model Prices'!$A$6:$I$15,4,FALSE)</x:f>
-        <x:v>0.1</x:v>
+        <x:v>0.02</x:v>
       </x:c>
       <x:c r="L15" s="249" t="n">
         <x:f>VLOOKUP(C15,'Model Prices'!$A$6:$I$15,6,FALSE)</x:f>
-        <x:v>6</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="M15" s="249" t="n">
         <x:f>VLOOKUP(C15,'Model Prices'!$A$6:$I$15,7,FALSE)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="N15" s="249" t="n">
         <x:f>VLOOKUP(C15,'Model Prices'!$A$6:$I$15,8,FALSE)</x:f>
-        <x:v>0.05</x:v>
+        <x:v>0.01</x:v>
       </x:c>
       <x:c r="O15" s="249" t="n">
         <x:f>VLOOKUP(C15,'Model Prices'!$A$6:$I$15,9,FALSE)</x:f>
-        <x:v>3</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="P15" s="249" t="n">
         <x:f>(E15*(1-F15)/'Assumptions'!$B$6)*(J15*(1-H15)+M15*H15)+(E15*F15/'Assumptions'!$B$6)*(K15*(1-H15)+N15*H15)+(G15/'Assumptions'!$B$6)*(L15*(1-H15)+O15*H15)</x:f>
-        <x:v>0.03495</x:v>
+        <x:v>0.00699</x:v>
       </x:c>
       <x:c r="Q15" s="249" t="n">
         <x:f>D15*I15*P15*(1+'Assumptions'!$B$13)*(1+'Assumptions'!$B$14)</x:f>
@@ -3884,35 +3884,35 @@
       </x:c>
       <x:c r="J16" s="249" t="n">
         <x:f>VLOOKUP(C16,'Model Prices'!$A$6:$I$15,3,FALSE)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="K16" s="249" t="n">
         <x:f>VLOOKUP(C16,'Model Prices'!$A$6:$I$15,4,FALSE)</x:f>
-        <x:v>0.1</x:v>
+        <x:v>0.02</x:v>
       </x:c>
       <x:c r="L16" s="249" t="n">
         <x:f>VLOOKUP(C16,'Model Prices'!$A$6:$I$15,6,FALSE)</x:f>
-        <x:v>6</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="M16" s="249" t="n">
         <x:f>VLOOKUP(C16,'Model Prices'!$A$6:$I$15,7,FALSE)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="N16" s="249" t="n">
         <x:f>VLOOKUP(C16,'Model Prices'!$A$6:$I$15,8,FALSE)</x:f>
-        <x:v>0.05</x:v>
+        <x:v>0.01</x:v>
       </x:c>
       <x:c r="O16" s="249" t="n">
         <x:f>VLOOKUP(C16,'Model Prices'!$A$6:$I$15,9,FALSE)</x:f>
-        <x:v>3</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="P16" s="249" t="n">
         <x:f>(E16*(1-F16)/'Assumptions'!$B$6)*(J16*(1-H16)+M16*H16)+(E16*F16/'Assumptions'!$B$6)*(K16*(1-H16)+N16*H16)+(G16/'Assumptions'!$B$6)*(L16*(1-H16)+O16*H16)</x:f>
-        <x:v>0.0143</x:v>
+        <x:v>0.00286</x:v>
       </x:c>
       <x:c r="Q16" s="249" t="n">
         <x:f>D16*I16*P16*(1+'Assumptions'!$B$13)*(1+'Assumptions'!$B$14)</x:f>
-        <x:v>0.000715</x:v>
+        <x:v>0.000143</x:v>
       </x:c>
       <x:c r="R16" s="241" t="str">
         <x:v>Luna low (human-authorized replacement for historical minimal); desired temperature 0 is not sent because compatibility with GPT-5.6 reasoning is not currently documented. Editable 5% structural-failure frequency.</x:v>
@@ -3937,7 +3937,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fb7b0348f0b49e5"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34db071a59314251"/>
 </x:worksheet>
 </file>
 
@@ -3996,7 +3996,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="124" t="str">
-        <x:v>Editable experiment assumptions. Model prices remain dated 2026-07-17; scenario results are planning estimates, not quotations.</x:v>
+        <x:v>Editable experiment assumptions. Luna prices observed 2026-08-08; scenario results are planning estimates, not quotations.</x:v>
       </x:c>
       <x:c r="B2" s="124"/>
       <x:c r="C2" s="124"/>
@@ -4022,7 +4022,7 @@
       </x:c>
       <x:c r="B3" s="133" t="n">
         <x:f>SUMIF('Call Profile'!$B$6:$B$16,"ACTIVITY",'Call Profile'!$Q$6:$Q$16)</x:f>
-        <x:v>0.5395025</x:v>
+        <x:v>0.0240205</x:v>
       </x:c>
       <x:c r="D3" s="159" t="str">
         <x:v>How to read: blue cells are editable scenario inputs; green cells are formulas. Models/tokens/cache/batch/escalation are edited by stage in Call Profile. Retry is edited in Assumptions. Technical/delivery excludes fixed infrastructure and human review; Total/delivery includes every modeled cost. Question scaling is a planning approximation until stage telemetry separates fixed and question-driven calls.</x:v>
@@ -4048,7 +4048,7 @@
       </x:c>
       <x:c r="B4" s="135" t="n">
         <x:f>SUMIF('Call Profile'!$B$6:$B$16,"SUBMISSION",'Call Profile'!$Q$6:$Q$16)</x:f>
-        <x:v>0.10517</x:v>
+        <x:v>0.021034</x:v>
       </x:c>
       <x:c r="D4" s="162"/>
       <x:c r="E4" s="163"/>
@@ -4238,11 +4238,11 @@
       </x:c>
       <x:c r="K10" s="209" t="n">
         <x:f>B10*$B$3</x:f>
-        <x:v>5.395025</x:v>
+        <x:v>0.240205</x:v>
       </x:c>
       <x:c r="L10" s="209" t="n">
         <x:f>E10*$B$4*(D10/$B$5)*(1+$B$6)</x:f>
-        <x:v>24.189099999999996</x:v>
+        <x:v>4.83782</x:v>
       </x:c>
       <x:c r="M10" s="209" t="n">
         <x:f>E10*F10*'Assumptions'!$B$8</x:f>
@@ -4262,11 +4262,11 @@
       </x:c>
       <x:c r="Q10" s="209" t="n">
         <x:f>SUM(J10:P10)+'Assumptions'!$B$15</x:f>
-        <x:v>496.4507916666667</x:v>
+        <x:v>471.9446916666667</x:v>
       </x:c>
       <x:c r="R10" s="214" t="n">
         <x:f>IF(E10=0,0,Q10/E10)</x:f>
-        <x:v>2.4822539583333336</x:v>
+        <x:v>2.3597234583333333</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26" customHeight="1">
@@ -4303,11 +4303,11 @@
       </x:c>
       <x:c r="K11" s="211" t="n">
         <x:f>B11*$B$3</x:f>
-        <x:v>2.6975125</x:v>
+        <x:v>0.1201025</x:v>
       </x:c>
       <x:c r="L11" s="211" t="n">
         <x:f>E11*$B$4*(D11/$B$5)*(1+$B$6)</x:f>
-        <x:v>18.141824999999997</x:v>
+        <x:v>3.6283649999999996</x:v>
       </x:c>
       <x:c r="M11" s="211" t="n">
         <x:f>E11*F11*'Assumptions'!$B$8</x:f>
@@ -4327,11 +4327,11 @@
       </x:c>
       <x:c r="Q11" s="211" t="n">
         <x:f>SUM(J11:P11)+'Assumptions'!$B$15</x:f>
-        <x:v>692.9393375</x:v>
+        <x:v>675.8484675</x:v>
       </x:c>
       <x:c r="R11" s="215" t="n">
         <x:f>IF(E11=0,0,Q11/E11)</x:f>
-        <x:v>4.619595583333333</x:v>
+        <x:v>4.50565645</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="26" customHeight="1">
@@ -4368,11 +4368,11 @@
       </x:c>
       <x:c r="K12" s="211" t="n">
         <x:f>B12*$B$3</x:f>
-        <x:v>10.79005</x:v>
+        <x:v>0.48041</x:v>
       </x:c>
       <x:c r="L12" s="211" t="n">
         <x:f>E12*$B$4*(D12/$B$5)*(1+$B$6)</x:f>
-        <x:v>241.891</x:v>
+        <x:v>48.37819999999999</x:v>
       </x:c>
       <x:c r="M12" s="211" t="n">
         <x:f>E12*F12*'Assumptions'!$B$8</x:f>
@@ -4392,11 +4392,11 @@
       </x:c>
       <x:c r="Q12" s="211" t="n">
         <x:f>SUM(J12:P12)+'Assumptions'!$B$15</x:f>
-        <x:v>5064.68105</x:v>
+        <x:v>4860.858609999999</x:v>
       </x:c>
       <x:c r="R12" s="215" t="n">
         <x:f>IF(E12=0,0,Q12/E12)</x:f>
-        <x:v>2.532340525</x:v>
+        <x:v>2.4304293049999997</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="26" customHeight="1">
@@ -4433,11 +4433,11 @@
       </x:c>
       <x:c r="K13" s="211" t="n">
         <x:f>B13*$B$3</x:f>
-        <x:v>53.95025</x:v>
+        <x:v>2.40205</x:v>
       </x:c>
       <x:c r="L13" s="211" t="n">
         <x:f>E13*$B$4*(D13/$B$5)*(1+$B$6)</x:f>
-        <x:v>2418.91</x:v>
+        <x:v>483.782</x:v>
       </x:c>
       <x:c r="M13" s="211" t="n">
         <x:f>E13*F13*'Assumptions'!$B$8</x:f>
@@ -4457,11 +4457,11 @@
       </x:c>
       <x:c r="Q13" s="211" t="n">
         <x:f>SUM(J13:P13)+'Assumptions'!$B$15</x:f>
-        <x:v>36099.52691666667</x:v>
+        <x:v>34112.85071666667</x:v>
       </x:c>
       <x:c r="R13" s="215" t="n">
         <x:f>IF(E13=0,0,Q13/E13)</x:f>
-        <x:v>1.8049763458333334</x:v>
+        <x:v>1.7056425358333334</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="26" customHeight="1">
@@ -4498,11 +4498,11 @@
       </x:c>
       <x:c r="K14" s="213" t="n">
         <x:f>B14*$B$3</x:f>
-        <x:v>107.9005</x:v>
+        <x:v>4.8041</x:v>
       </x:c>
       <x:c r="L14" s="213" t="n">
         <x:f>E14*$B$4*(D14/$B$5)*(1+$B$6)</x:f>
-        <x:v>12094.55</x:v>
+        <x:v>2418.91</x:v>
       </x:c>
       <x:c r="M14" s="213" t="n">
         <x:f>E14*F14*'Assumptions'!$B$8</x:f>
@@ -4522,11 +4522,11 @@
       </x:c>
       <x:c r="Q14" s="213" t="n">
         <x:f>SUM(J14:P14)+'Assumptions'!$B$15</x:f>
-        <x:v>139869.11716666666</x:v>
+        <x:v>130090.38076666667</x:v>
       </x:c>
       <x:c r="R14" s="216" t="n">
         <x:f>IF(E14=0,0,Q14/E14)</x:f>
-        <x:v>1.3986911716666666</x:v>
+        <x:v>1.3009038076666666</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -4565,7 +4565,7 @@
       </x:c>
       <x:c r="U22" s="226" t="n">
         <x:f>IF(E10=0,0,(K10+L10)/E10)</x:f>
-        <x:v>0.14792062499999997</x:v>
+        <x:v>0.025390125</x:v>
       </x:c>
       <x:c r="V22" s="226" t="n">
         <x:f>IF(E10=0,0,(M10+N10+O10)/E10)</x:f>
@@ -4581,11 +4581,11 @@
       </x:c>
       <x:c r="Y22" s="232" t="n">
         <x:f>IF(E10=0,0,(K10+L10+M10+N10+O10)/E10)</x:f>
-        <x:v>0.14892062499999997</x:v>
+        <x:v>0.026390125</x:v>
       </x:c>
       <x:c r="Z22" s="235" t="n">
         <x:f>R10</x:f>
-        <x:v>2.4822539583333336</x:v>
+        <x:v>2.3597234583333333</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -4598,7 +4598,7 @@
       </x:c>
       <x:c r="U23" s="228" t="n">
         <x:f>IF(E11=0,0,(K11+L11)/E11)</x:f>
-        <x:v>0.13892891666666665</x:v>
+        <x:v>0.024989783333333328</x:v>
       </x:c>
       <x:c r="V23" s="228" t="n">
         <x:f>IF(E11=0,0,(M11+N11+O11)/E11)</x:f>
@@ -4614,11 +4614,11 @@
       </x:c>
       <x:c r="Y23" s="233" t="n">
         <x:f>IF(E11=0,0,(K11+L11+M11+N11+O11)/E11)</x:f>
-        <x:v>0.20292891666666668</x:v>
+        <x:v>0.08898978333333332</x:v>
       </x:c>
       <x:c r="Z23" s="236" t="n">
         <x:f>R11</x:f>
-        <x:v>4.619595583333333</x:v>
+        <x:v>4.50565645</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -4631,7 +4631,7 @@
       </x:c>
       <x:c r="U24" s="228" t="n">
         <x:f>IF(E12=0,0,(K12+L12)/E12)</x:f>
-        <x:v>0.126340525</x:v>
+        <x:v>0.024429304999999995</x:v>
       </x:c>
       <x:c r="V24" s="228" t="n">
         <x:f>IF(E12=0,0,(M12+N12+O12)/E12)</x:f>
@@ -4647,11 +4647,11 @@
       </x:c>
       <x:c r="Y24" s="233" t="n">
         <x:f>IF(E12=0,0,(K12+L12+M12+N12+O12)/E12)</x:f>
-        <x:v>0.182340525</x:v>
+        <x:v>0.08042930499999999</x:v>
       </x:c>
       <x:c r="Z24" s="236" t="n">
         <x:f>R12</x:f>
-        <x:v>2.532340525</x:v>
+        <x:v>2.4304293049999997</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -4664,7 +4664,7 @@
       </x:c>
       <x:c r="U25" s="228" t="n">
         <x:f>IF(E13=0,0,(K13+L13)/E13)</x:f>
-        <x:v>0.12364301249999998</x:v>
+        <x:v>0.024309202499999998</x:v>
       </x:c>
       <x:c r="V25" s="228" t="n">
         <x:f>IF(E13=0,0,(M13+N13+O13)/E13)</x:f>
@@ -4680,11 +4680,11 @@
       </x:c>
       <x:c r="Y25" s="233" t="n">
         <x:f>IF(E13=0,0,(K13+L13+M13+N13+O13)/E13)</x:f>
-        <x:v>0.1716430125</x:v>
+        <x:v>0.07230920249999999</x:v>
       </x:c>
       <x:c r="Z25" s="236" t="n">
         <x:f>R13</x:f>
-        <x:v>1.8049763458333334</x:v>
+        <x:v>1.7056425358333334</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -4694,7 +4694,7 @@
       </x:c>
       <x:c r="U26" s="230" t="n">
         <x:f>IF(E14=0,0,(K14+L14)/E14)</x:f>
-        <x:v>0.12202450499999999</x:v>
+        <x:v>0.024237140999999997</x:v>
       </x:c>
       <x:c r="V26" s="230" t="n">
         <x:f>IF(E14=0,0,(M14+N14+O14)/E14)</x:f>
@@ -4710,11 +4710,11 @@
       </x:c>
       <x:c r="Y26" s="234" t="n">
         <x:f>IF(E14=0,0,(K14+L14+M14+N14+O14)/E14)</x:f>
-        <x:v>0.16202450499999999</x:v>
+        <x:v>0.064237141</x:v>
       </x:c>
       <x:c r="Z26" s="237" t="n">
         <x:f>R14</x:f>
-        <x:v>1.3986911716666666</x:v>
+        <x:v>1.3009038076666666</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4748,8 +4748,8 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racc271c39f2740b9"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45b7b6519a794c43"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9891ead7809416b"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8d6175429944d63"/>
 </x:worksheet>
 </file>
 
@@ -5450,7 +5450,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>The resolver applies approved configurations; it does not choose the 'best model' dynamically. Capabilities and data policy are checked before every call.</x:v>
+        <x:v>Active route profile: LUNA_BASELINE_V1. It is deterministic, Luna-only, has no fallback or heuristic selection, and preserves the mixed Sol/Luna profile only as history.</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
         <x:v>Primary routes are a hypothesis to validate on the institutional golden set. Quality and privacy gates override price; model snapshots must be pinned where the provider supports it.</x:v>
@@ -5479,7 +5479,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="7" t="str">
-        <x:v>Primary routes are a hypothesis to validate on the institutional golden set. Quality and privacy gates override price; model snapshots must be pinned where the provider supports it.</x:v>
+        <x:v>Active route profile: LUNA_BASELINE_V1. It is deterministic, Luna-only, has no fallback or heuristic selection, and preserves the mixed Sol/Luna profile only as history.</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
         <x:v>Primary routes are a hypothesis to validate on the institutional golden set. Quality and privacy gates override price; model snapshots must be pinned where the provider supports it.</x:v>
@@ -5540,7 +5540,7 @@
         <x:v>P01 Activity spec</x:v>
       </x:c>
       <x:c r="B6" s="29" t="str">
-        <x:v>GPT-5.6 Sol</x:v>
+        <x:v>GPT-5.6 Luna</x:v>
       </x:c>
       <x:c r="C6" s="29" t="str">
         <x:v>medium</x:v>
@@ -5552,7 +5552,7 @@
         <x:v>Text + structured JSON</x:v>
       </x:c>
       <x:c r="F6" s="29" t="str">
-        <x:v>Approved route only</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="G6" s="29" t="str">
         <x:v>No dynamic escalation</x:v>
@@ -5569,7 +5569,7 @@
         <x:v>P02 Rubric normalize</x:v>
       </x:c>
       <x:c r="B7" s="29" t="str">
-        <x:v>GPT-5.6 Sol</x:v>
+        <x:v>GPT-5.6 Luna</x:v>
       </x:c>
       <x:c r="C7" s="29" t="str">
         <x:v>medium</x:v>
@@ -5581,7 +5581,7 @@
         <x:v>Text + structured JSON</x:v>
       </x:c>
       <x:c r="F7" s="29" t="str">
-        <x:v>Approved route only</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="G7" s="29" t="str">
         <x:v>No dynamic escalation</x:v>
@@ -5610,7 +5610,7 @@
         <x:v>Text + structured JSON</x:v>
       </x:c>
       <x:c r="F8" s="29" t="str">
-        <x:v>Human review</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="G8" s="29" t="str">
         <x:v>Mapping uncertainty or policy issue</x:v>
@@ -5627,7 +5627,7 @@
         <x:v>P04 Blueprint build</x:v>
       </x:c>
       <x:c r="B9" s="29" t="str">
-        <x:v>GPT-5.6 Sol</x:v>
+        <x:v>GPT-5.6 Luna</x:v>
       </x:c>
       <x:c r="C9" s="29" t="str">
         <x:v>high</x:v>
@@ -5639,7 +5639,7 @@
         <x:v>Long text + structured JSON</x:v>
       </x:c>
       <x:c r="F9" s="29" t="str">
-        <x:v>Approved route only</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="G9" s="29" t="str">
         <x:v>Critical P05 correction</x:v>
@@ -5656,7 +5656,7 @@
         <x:v>P05 Blueprint review</x:v>
       </x:c>
       <x:c r="B10" s="29" t="str">
-        <x:v>GPT-5.6 Sol</x:v>
+        <x:v>GPT-5.6 Luna</x:v>
       </x:c>
       <x:c r="C10" s="29" t="str">
         <x:v>high</x:v>
@@ -5668,7 +5668,7 @@
         <x:v>Long text + structured JSON</x:v>
       </x:c>
       <x:c r="F10" s="29" t="str">
-        <x:v>Human review</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="G10" s="29" t="str">
         <x:v>Critical FAIL</x:v>
@@ -5697,7 +5697,7 @@
         <x:v>Text/image crop + structured JSON</x:v>
       </x:c>
       <x:c r="F11" s="29" t="str">
-        <x:v>Review/block</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="G11" s="29" t="str">
         <x:v>Low extraction confidence, insufficient detail, complex relation</x:v>
@@ -5726,7 +5726,7 @@
         <x:v>Text/image crop + structured JSON</x:v>
       </x:c>
       <x:c r="F12" s="29" t="str">
-        <x:v>Reserve opportunity</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="G12" s="29" t="str">
         <x:v>Validation failure; no model/provider widening</x:v>
@@ -5755,7 +5755,7 @@
         <x:v>Text/image crop + structured JSON</x:v>
       </x:c>
       <x:c r="F13" s="29" t="str">
-        <x:v>Human review</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="G13" s="29" t="str">
         <x:v>Genuine ambiguity only</x:v>
@@ -5784,7 +5784,7 @@
         <x:v>Structured JSON</x:v>
       </x:c>
       <x:c r="F14" s="29" t="str">
-        <x:v>Human review</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="G14" s="29" t="str">
         <x:v>Unsupported observable guide</x:v>
@@ -5842,7 +5842,7 @@
         <x:v>Structured JSON</x:v>
       </x:c>
       <x:c r="F16" s="29" t="str">
-        <x:v>Review/block</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="G16" s="29" t="str">
         <x:v>Exactly one structural attempt</x:v>
@@ -5885,28 +5885,28 @@
     </x:row>
     <x:row r="18" ht="68" customHeight="1">
       <x:c r="A18" s="73" t="str">
-        <x:v>Terra policy</x:v>
+        <x:v>Historical mixed Sol/Luna</x:v>
       </x:c>
       <x:c r="B18" s="32" t="str">
-        <x:v>Not callable in this gate</x:v>
+        <x:v>P01/P02/P04/P05 Sol; other callable prompts Luna</x:v>
       </x:c>
       <x:c r="C18" s="32" t="str">
-        <x:v>n/a</x:v>
+        <x:v>Comparison only</x:v>
       </x:c>
       <x:c r="D18" s="32" t="str">
         <x:v>not sent</x:v>
       </x:c>
       <x:c r="E18" s="32" t="str">
-        <x:v>Historical reference only</x:v>
+        <x:v>Historical route profile</x:v>
       </x:c>
       <x:c r="F18" s="32" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="G18" s="32" t="str">
-        <x:v>No eligibility in this gate</x:v>
+        <x:v>Not callable; future human authorization required</x:v>
       </x:c>
       <x:c r="H18" s="32" t="str">
-        <x:v>Terra excluded by the binding route matrix</x:v>
+        <x:v>No automatic fallback to Sol</x:v>
       </x:c>
       <x:c r="I18" s="32" t="str">
         <x:v>No evaluation in this gate</x:v>
@@ -6015,10 +6015,10 @@
         <x:v>https://developers.openai.com/api/docs/pricing</x:v>
       </x:c>
       <x:c r="D6" s="29" t="str">
-        <x:v>2026-07-17</x:v>
+        <x:v>2026-08-08</x:v>
       </x:c>
       <x:c r="E6" s="29" t="str">
-        <x:v>Sol/Terra/Luna standard, cache, batch and regional/long-context notes.</x:v>
+        <x:v>Luna Standard short-context 0.20/0.02/0.25/1.20; Batch 0.10/0.01/0.125/0.60. Recheck before spend.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="52" customHeight="1">

</xml_diff>